<commit_message>
Fix Soroti + live run-demo + all Uganda visible
- scraper.py: add scrape_soroti() for https://sun.ac.ug/staff-directory/ (77 records), fix URLs for MUST/Kyambogo, fast CoCIS
- input/Universities.csv: correct Soroti URL, remove duplicate, fix MUST/Kyambogo URLs
- app.py: run-demo now spawns background thread (actual scrape), pagination 20/page fixes endless load, data_source dynamic
- output: 246 records from 8/43 (Makerere 145, Soroti 77, Gulu 5, etc.)
</commit_message>
<xml_diff>
--- a/output/universities.xlsx
+++ b/output/universities.xlsx
@@ -413,12 +413,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G170"/>
+  <dimension ref="A1:G247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="82" customWidth="1" min="4" max="4"/>
     <col width="85" customWidth="1" min="5" max="5"/>
     <col width="105" customWidth="1" min="6" max="6"/>
@@ -5575,28 +5575,32 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Islamic University In Uganda</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>SponsorCentenary BankSupporting the 5th Edition of Run for Girl Child Education.</t>
-        </is>
-      </c>
-      <c r="E152" t="inlineStr"/>
+          <t>Dr. Kirya Fred</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Associate Professor/Dean SHS/ Senate Rep. To Council</t>
+        </is>
+      </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>assets/images/home/run4girl-sponsors/centenary-bank.jpg</t>
+          <t>Image not Found</t>
         </is>
       </c>
       <c r="G152" t="inlineStr"/>
@@ -5604,28 +5608,32 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Islamic University In Uganda</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Hydration PartnerZora WaterOfficial Hydration Partner for the 5th Edition.</t>
-        </is>
-      </c>
-      <c r="E153" t="inlineStr"/>
+          <t>Dr. Othieno Emmanuel</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>assets/images/home/run4girl-sponsors/zora-water.jpg</t>
+          <t>Image not Found</t>
         </is>
       </c>
       <c r="G153" t="inlineStr"/>
@@ -5633,28 +5641,32 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Islamic University In Uganda</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>SponsorSplash KachupaJoining the run for brighter futures and stronger dreams.</t>
-        </is>
-      </c>
-      <c r="E154" t="inlineStr"/>
+          <t>Dr. Ntale Roman Saba</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>assets/images/home/run4girl-sponsors/splash-kachupa.jpg</t>
+          <t>Image not Found</t>
         </is>
       </c>
       <c r="G154" t="inlineStr"/>
@@ -5662,28 +5674,32 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Islamic University In Uganda</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Proud SupporterTropical BankHelping keep girls in school through every step.</t>
-        </is>
-      </c>
-      <c r="E155" t="inlineStr"/>
+          <t>Dr. Aderu David</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Senior Lecturer</t>
+        </is>
+      </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>assets/images/home/run4girl-sponsors/tropical-bank.jpg</t>
+          <t>Image not Found</t>
         </is>
       </c>
       <c r="G155" t="inlineStr"/>
@@ -5691,27 +5707,27 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Islamic University In Uganda</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Academic Calendar</t>
+          <t>Dr. Katongole Paul</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Senior Lecturer</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -5724,27 +5740,27 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Islamic University In Uganda</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Alumni Affairs</t>
+          <t>Dr. Winifred Nabwire Wafula</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Senior Lecturer</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -5757,27 +5773,27 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Islamic University In Uganda</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Council</t>
+          <t>Dr. Eleku Simon</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Senior Lecturer</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -5790,27 +5806,27 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Uganda Pentecostal University</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Quick Links</t>
+          <t>Dr. Richard Mpango</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Senior Lecturer</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -5823,27 +5839,27 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Uganda Pentecostal University</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>UPU E-system</t>
+          <t>Dr. Kabwigu Samuel</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Senior Lecturer</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -5856,27 +5872,27 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Uganda Pentecostal University</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Get In Touch</t>
+          <t>Dr. Amuron Naomi</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Lecturer</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -5889,28 +5905,32 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Iuiu Mbale</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>SponsorCentenary BankSupporting the 5th Edition of Run for Girl Child Education.</t>
-        </is>
-      </c>
-      <c r="E162" t="inlineStr"/>
+          <t>Dr. Luwede Aliba Flavia</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>assets/images/home/run4girl-sponsors/centenary-bank.jpg</t>
+          <t>Image not Found</t>
         </is>
       </c>
       <c r="G162" t="inlineStr"/>
@@ -5918,28 +5938,32 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Iuiu Mbale</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Hydration PartnerZora WaterOfficial Hydration Partner for the 5th Edition.</t>
-        </is>
-      </c>
-      <c r="E163" t="inlineStr"/>
+          <t>Dr. Olupot Robert</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>assets/images/home/run4girl-sponsors/zora-water.jpg</t>
+          <t>Image not Found</t>
         </is>
       </c>
       <c r="G163" t="inlineStr"/>
@@ -5947,28 +5971,32 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Iuiu Mbale</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>SponsorSplash KachupaJoining the run for brighter futures and stronger dreams.</t>
-        </is>
-      </c>
-      <c r="E164" t="inlineStr"/>
+          <t>Mr. Mwesige Samuel</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>assets/images/home/run4girl-sponsors/splash-kachupa.jpg</t>
+          <t>Image not Found</t>
         </is>
       </c>
       <c r="G164" t="inlineStr"/>
@@ -5976,28 +6004,32 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Iuiu Mbale</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Proud SupporterTropical BankHelping keep girls in school through every step.</t>
-        </is>
-      </c>
-      <c r="E165" t="inlineStr"/>
+          <t>Mr. Munguiko Clement</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>assets/images/home/run4girl-sponsors/tropical-bank.jpg</t>
+          <t>Image not Found</t>
         </is>
       </c>
       <c r="G165" t="inlineStr"/>
@@ -6005,27 +6037,27 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Iuiu Mbale</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Academic Calendar</t>
+          <t>Mr. Kateregga James</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Lecturer</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -6038,27 +6070,27 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Iuiu Mbale</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Alumni Affairs</t>
+          <t>Mr. Otim Paul</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Lecturer</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -6071,27 +6103,27 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Iuiu Mbale</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Council</t>
+          <t>Ms. Nabusige Jean Brenda Gesa</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Lecturer</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -6104,27 +6136,27 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Ankole Western University</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Soroti University</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Auto-detected</t>
+          <t>Staff Directory</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>1st Graduation List for the 7th Graduation Ceremony of AWU 2024</t>
+          <t>Mr. Emmanuel Denis Morgan Thomas</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Tuhairwe shiberah</t>
+          <t>Lecturer</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -6137,35 +6169,2544 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Dr. Namwase Hadijja Katabira</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Dr. Abwola Mary Olwedo</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Mr. Ojakol Alex Imalingat</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Ms. Kiconco Ritah</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Dr. Bahati Johnson</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Dr. Kirya Musa</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Dr. Opito Ronald</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Dr. Engoru Ejoru Charles</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Mr. Kizito Mark</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Mr. Yahaya Joseph James</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Ms. Atim Letizia</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Ms. Namujju Josephine</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Mr. Atukwatse Joseph</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Ms. Nankinga Clare</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Dr. Okuja Maxwell</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Mr. Aneth Ephrem Gregory</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Mr. Okello Samuel</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Mr. Okoboi Joash</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Dr. Lwere Kamada</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Mr. Kiguli James Mukasa</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Assistant Lecturer</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Mr. Adakun Moses</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Assistant Lecturer</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Dr. Odongo Charles Newton</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Assistant Lecturer</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Mr. Kizito Mary Muwonge</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Assistant Lecturer</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Mr. Kinobe Robert</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Assistant Lecturer</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Ms. Nakalembe Loyce</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Assistant Lecturer</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Mr. Ayikobua Emmanuel Tiyo</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Assistant Lecturer/ Academic Staff Rep To Council</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Dr. Cherop Moses</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Assistant Lecturer</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Ms. Akurut Hellen</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Assistant Lecturer</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Dr. Lubogo Patrick</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Assistant Lecturer</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Dr. Kyegombe William</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Assistant Lecturer</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Dr. Apolot Denis</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Assistant Lecturer</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Mr. Nkangi Lwanga Eriasaph</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Chief Technician</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Ms. Apolot Esther</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Lab Attendant</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Ms. Cheptoek Sarah Musani</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Lab Technician</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Mr. Aculet Valentine</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Laboratory Technician</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Ms. Akello Safina</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Skills Lab Instructor</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Mr. Apedel Micheal</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Lab Attendant</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Mr. Baguma Kenneth</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Lab Technician</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Mr. Etanu Simon</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Lab Attendant</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Mr. Malinga Gerald Patrick</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Lab Assistant</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Mr. Musilimu Pamba</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Laboratory Technician</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Ms. Nabwire Sandra</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Science Laboratory Assistant</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Mr. Nuwamanya Newton</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Laboratory Technician</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Mr. Ocan Samuel</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Laboratory Technician</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Mr. Ojuko Samuel</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Laboratory Technician</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Mr. Ojula Emmanuel</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Lab Attendant</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Mr. Opiding Francis</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Laboratory Technician</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Mr. Opio James Peter</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Lab Attendant</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Mr. Otim Jimmy Shadrack</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Lab Assistant</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Mr. Ruhangariyo Robert</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Lab Technician</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Ms. Awino Mariam Abdallah</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Assistant Administrator</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Mr. Sengendo Geofrey</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Academic Staff</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Mr. Ahimbisibwe Octavious</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Technician</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Ms. Mone Tina</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Senior Administrator</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Mr. Epou Solomon</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Office Assistant</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Mr. Osuwat Lawrence Obado</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Academic Staff</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Student Services</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Academic Staff</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Academics</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Academic Staff</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Soroti University</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Staff Directory</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Useful Links</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Academic Staff</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Islamic University In Uganda</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>SponsorCentenary BankSupporting the 5th Edition of Run for Girl Child Education.</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr"/>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>assets/images/home/run4girl-sponsors/centenary-bank.jpg</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Islamic University In Uganda</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Hydration PartnerZora WaterOfficial Hydration Partner for the 5th Edition.</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr"/>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>assets/images/home/run4girl-sponsors/zora-water.jpg</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Islamic University In Uganda</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>SponsorSplash KachupaJoining the run for brighter futures and stronger dreams.</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr"/>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>assets/images/home/run4girl-sponsors/splash-kachupa.jpg</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Islamic University In Uganda</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Proud SupporterTropical BankHelping keep girls in school through every step.</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr"/>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>assets/images/home/run4girl-sponsors/tropical-bank.jpg</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Islamic University In Uganda</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Academic Calendar</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Islamic University In Uganda</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Alumni Affairs</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Islamic University In Uganda</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Council</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Uganda Pentecostal University</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Quick Links</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr"/>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Uganda Pentecostal University</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>UPU E-system</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Uganda Pentecostal University</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Get In Touch</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Iuiu Mbale</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>SponsorCentenary BankSupporting the 5th Edition of Run for Girl Child Education.</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr"/>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>assets/images/home/run4girl-sponsors/centenary-bank.jpg</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Iuiu Mbale</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Hydration PartnerZora WaterOfficial Hydration Partner for the 5th Edition.</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr"/>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>assets/images/home/run4girl-sponsors/zora-water.jpg</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Iuiu Mbale</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>SponsorSplash KachupaJoining the run for brighter futures and stronger dreams.</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr"/>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>assets/images/home/run4girl-sponsors/splash-kachupa.jpg</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Iuiu Mbale</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Proud SupporterTropical BankHelping keep girls in school through every step.</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr"/>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>assets/images/home/run4girl-sponsors/tropical-bank.jpg</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Iuiu Mbale</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Academic Calendar</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Iuiu Mbale</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Alumni Affairs</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Iuiu Mbale</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Council</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
           <t>Ankole Western University</t>
         </is>
       </c>
-      <c r="B170" t="inlineStr">
+      <c r="B246" t="inlineStr">
         <is>
           <t>Auto-detected</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr">
+      <c r="C246" t="inlineStr">
         <is>
           <t>Auto-detected</t>
         </is>
       </c>
-      <c r="D170" t="inlineStr">
+      <c r="D246" t="inlineStr">
         <is>
           <t>1st Graduation List for the 7th Graduation Ceremony of AWU 2024</t>
         </is>
       </c>
-      <c r="E170" t="inlineStr">
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Tuhairwe shiberah</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Ankole Western University</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Auto-detected</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>1st Graduation List for the 7th Graduation Ceremony of AWU 2024</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
         <is>
           <t>Katungwensi Derick</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr">
-        <is>
-          <t>Image not Found</t>
-        </is>
-      </c>
-      <c r="G170" t="inlineStr"/>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Image not Found</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>